<commit_message>
Restarted docs and added unit tests for missing modules
</commit_message>
<xml_diff>
--- a/download_results.xlsx
+++ b/download_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f19994348ecc0c8c/Documents/GitHub/biomarkit/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackb\OneDrive\Documents\GitHub\biomarkit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="109" documentId="8_{0A07A6D1-C489-484C-B36E-41B1081D4BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A26365B-252E-41ED-92E8-8613A680176E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77E613F-EF9E-408B-8144-9D7FA0177B89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21900" yWindow="108" windowWidth="19272" windowHeight="16452" activeTab="1" xr2:uid="{8F929425-8DF4-4B26-B085-8A7345256B39}"/>
+    <workbookView xWindow="49920" yWindow="6048" windowWidth="19272" windowHeight="16452" activeTab="1" xr2:uid="{8F929425-8DF4-4B26-B085-8A7345256B39}"/>
   </bookViews>
   <sheets>
     <sheet name="1.A" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="16">
   <si>
     <t>biomarkit</t>
   </si>
@@ -85,6 +85,9 @@
   </si>
   <si>
     <t>standardise()</t>
+  </si>
+  <si>
+    <t>Transform() CPU</t>
   </si>
 </sst>
 </file>
@@ -155,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -170,6 +173,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -632,7 +636,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9D3FD84-E77C-45DA-BE9E-65531FBC0B6F}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
@@ -665,29 +669,43 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="5">
-        <v>4530</v>
-      </c>
-      <c r="C3" s="5">
-        <v>4782</v>
-      </c>
-      <c r="D3" s="5">
-        <v>5139</v>
+        <v>15</v>
+      </c>
+      <c r="B3" s="8">
+        <v>6478</v>
+      </c>
+      <c r="C3" s="8">
+        <v>10611</v>
+      </c>
+      <c r="D3" s="8">
+        <v>6885</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="5">
+        <v>4530</v>
+      </c>
+      <c r="C4" s="5">
+        <v>4782</v>
+      </c>
+      <c r="D4" s="5">
+        <v>5139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B5" s="5">
         <v>760</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C5" s="5">
         <v>1741</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D5" s="5">
         <v>846</v>
       </c>
     </row>

</xml_diff>